<commit_message>
semana 8 de 2026 , con ajustes en circulacion viral de 2026.
</commit_message>
<xml_diff>
--- a/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
+++ b/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -371,7 +371,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>580</v>
+        <v>608</v>
       </c>
     </row>
     <row r="3">
@@ -379,7 +379,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>548</v>
+        <v>498</v>
       </c>
     </row>
     <row r="4">
@@ -387,7 +387,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>549</v>
+        <v>553</v>
       </c>
     </row>
     <row r="5">
@@ -395,7 +395,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>395</v>
+        <v>369</v>
       </c>
     </row>
     <row r="6">
@@ -403,7 +403,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>499</v>
+        <v>511</v>
       </c>
     </row>
     <row r="7">
@@ -411,7 +411,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>451</v>
+        <v>509</v>
       </c>
     </row>
     <row r="8">
@@ -419,7 +419,23 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>56</v>
+        <v>527</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
semana 09 de 2026
</commit_message>
<xml_diff>
--- a/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
+++ b/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -427,7 +427,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>414</v>
+        <v>456</v>
       </c>
     </row>
     <row r="10">
@@ -435,7 +435,15 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>3</v>
+        <v>728</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
semana 10 de 2026
</commit_message>
<xml_diff>
--- a/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
+++ b/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -371,7 +371,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>608</v>
+        <v>633</v>
       </c>
     </row>
     <row r="3">
@@ -387,7 +387,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>553</v>
+        <v>571</v>
       </c>
     </row>
     <row r="5">
@@ -395,7 +395,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>369</v>
+        <v>398</v>
       </c>
     </row>
     <row r="6">
@@ -411,7 +411,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="8">
@@ -419,7 +419,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>527</v>
+        <v>524</v>
       </c>
     </row>
     <row r="9">
@@ -427,7 +427,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>456</v>
+        <v>450</v>
       </c>
     </row>
     <row r="10">
@@ -435,7 +435,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>728</v>
+        <v>435</v>
       </c>
     </row>
     <row r="11">
@@ -443,7 +443,15 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>10</v>
+        <v>384</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
semana 12 de 2026
</commit_message>
<xml_diff>
--- a/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
+++ b/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -371,7 +371,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>633</v>
+        <v>618</v>
       </c>
     </row>
     <row r="3">
@@ -419,7 +419,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>524</v>
+        <v>504</v>
       </c>
     </row>
     <row r="9">
@@ -443,7 +443,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>384</v>
+        <v>426</v>
       </c>
     </row>
     <row r="12">
@@ -451,7 +451,23 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>29</v>
+        <v>485</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Semana 13 de 2026
</commit_message>
<xml_diff>
--- a/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
+++ b/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -467,7 +467,15 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>21</v>
+        <v>367</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
semana 14 pasada, y de esta semana subi epi1,2,3 por que por git hub directo no pude
</commit_message>
<xml_diff>
--- a/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
+++ b/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
@@ -443,7 +443,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>426</v>
+        <v>456</v>
       </c>
     </row>
     <row r="12">
@@ -451,7 +451,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>485</v>
+        <v>488</v>
       </c>
     </row>
     <row r="13">
@@ -459,7 +459,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>564</v>
+        <v>551</v>
       </c>
     </row>
     <row r="14">
@@ -467,7 +467,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>367</v>
+        <v>404</v>
       </c>
     </row>
     <row r="15">
@@ -475,7 +475,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>33</v>
+        <v>505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
semana 15 de 2026
</commit_message>
<xml_diff>
--- a/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
+++ b/Boletin_ Epi_Pereira/Datos/eda2018.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -475,7 +475,23 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>505</v>
+        <v>559</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>